<commit_message>
Publish fixed boss pack artifacts
</commit_message>
<xml_diff>
--- a/boss_pack/company_count_evidence.xlsx
+++ b/boss_pack/company_count_evidence.xlsx
@@ -1077,7 +1077,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>https://github.com/RnDprincipiacapital/SME-Dual_Engine/blob/main/samples/galway-sme-dashboard-expanded-public.json</t>
+          <t>https://rndprincipiacapital.github.io/sme-dual-engine-public/targets.json</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>https://github.com/RnDprincipiacapital/SME-Dual_Engine/blob/main/samples/galway-sme-dashboard-expanded-public.json</t>
+          <t>https://rndprincipiacapital.github.io/sme-dual-engine-public/targets.json</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>https://github.com/RnDprincipiacapital/SME-Dual_Engine/blob/main/samples/galway-sme-dashboard-expanded-public.json</t>
+          <t>https://rndprincipiacapital.github.io/sme-dual-engine-public/targets.json</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>https://github.com/RnDprincipiacapital/SME-Dual_Engine/blob/main/samples/galway-sme-dashboard-expanded-public.json</t>
+          <t>https://rndprincipiacapital.github.io/sme-dual-engine-public/targets.json</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>https://github.com/RnDprincipiacapital/SME-Dual_Engine/blob/main/samples/galway-sme-dashboard-expanded-public.json</t>
+          <t>https://rndprincipiacapital.github.io/sme-dual-engine-public/targets.json</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>https://github.com/RnDprincipiacapital/SME-Dual_Engine/blob/main/samples/galway-sme-dashboard-expanded-public.json</t>
+          <t>https://rndprincipiacapital.github.io/sme-dual-engine-public/targets.json</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">

</xml_diff>